<commit_message>
Edited BasePage created new Page PracticeFormPage,Added new sheet on test data, Created new Test Case for Form
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joyia\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8A936D-2B89-43C4-8F2D-7FE886C5E545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58439DE5-9DCB-4948-A54A-B294E43E9ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Forms" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>UserName</t>
   </si>
@@ -49,16 +50,60 @@
   </si>
   <si>
     <t>Password123</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>UserNumber</t>
+  </si>
+  <si>
+    <t>DateOfBirth</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>10 Apr 1999</t>
+  </si>
+  <si>
+    <t>1234567890</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>test@mailinator.com</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Doe</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -81,14 +126,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -475,4 +523,65 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E8F5D29-B261-4791-A884-F5DFAD0642EF}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="2" width="9.06640625" style="1"/>
+    <col min="3" max="3" width="17.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.06640625" style="1"/>
+    <col min="5" max="5" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.9296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.06640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{6570131B-F6A1-4AD3-82A7-02314EC3CC99}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added New Element FileUpload and Dropdown selector.
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joyia\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58439DE5-9DCB-4948-A54A-B294E43E9ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF0D248-4C62-4A4E-8C0E-3C4DC9430E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="16200" windowHeight="9308" activeTab="2" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t>UserName</t>
   </si>
@@ -86,6 +86,24 @@
   </si>
   <si>
     <t>Doe</t>
+  </si>
+  <si>
+    <t>fileInput</t>
+  </si>
+  <si>
+    <t>src/main/resources/testdata/sample.jpg</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>NCR</t>
+  </si>
+  <si>
+    <t>Delhi</t>
   </si>
 </sst>
 </file>
@@ -527,7 +545,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E8F5D29-B261-4791-A884-F5DFAD0642EF}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="9.06640625" style="1"/>
@@ -535,10 +553,11 @@
     <col min="4" max="4" width="9.06640625" style="1"/>
     <col min="5" max="5" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.9296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.06640625" style="1"/>
+    <col min="7" max="7" width="32.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -557,8 +576,17 @@
       <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -576,6 +604,15 @@
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added New Element Checkbox which checks Labels and Value
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joyia\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF0D248-4C62-4A4E-8C0E-3C4DC9430E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3207E60C-352E-4548-831A-3387C7AAC85E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1470" yWindow="1470" windowWidth="16200" windowHeight="9308" activeTab="2" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>UserName</t>
   </si>
@@ -104,6 +104,12 @@
   </si>
   <si>
     <t>Delhi</t>
+  </si>
+  <si>
+    <t>Hobbies</t>
+  </si>
+  <si>
+    <t>Music,Sports</t>
   </si>
 </sst>
 </file>
@@ -545,7 +551,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E8F5D29-B261-4791-A884-F5DFAD0642EF}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="9.06640625" style="1"/>
@@ -557,7 +563,7 @@
     <col min="8" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -585,8 +591,11 @@
       <c r="I1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -613,6 +622,9 @@
       </c>
       <c r="I2" s="1" t="s">
         <v>21</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added AlertsFramesModals page. Added Handling for new tabs in the base page class. Created a new Test Case for Alerts
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joyia\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3207E60C-352E-4548-831A-3387C7AAC85E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB642C-9BF7-47C6-9519-678BE645CAA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="16200" windowHeight="9308" activeTab="2" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Forms" sheetId="3" r:id="rId3"/>
+    <sheet name="Alerts" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>UserName</t>
   </si>
@@ -110,6 +111,12 @@
   </si>
   <si>
     <t>Music,Sports</t>
+  </si>
+  <si>
+    <t>SampleHeading</t>
+  </si>
+  <si>
+    <t>This is a sample page</t>
   </si>
 </sst>
 </file>
@@ -633,4 +640,27 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5090DDF-4D7E-44B7-9BA1-7EC99A42EFDA}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="17.1328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added new Test Case for Alert added Alerts handling on basePage
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joyia\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB642C-9BF7-47C6-9519-678BE645CAA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{996C355D-9F1F-4209-A877-37F7C38FCB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>UserName</t>
   </si>
@@ -117,6 +117,12 @@
   </si>
   <si>
     <t>This is a sample page</t>
+  </si>
+  <si>
+    <t>ASD@#@123</t>
+  </si>
+  <si>
+    <t>Prompt</t>
   </si>
 </sst>
 </file>
@@ -644,23 +650,33 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5090DDF-4D7E-44B7-9BA1-7EC99A42EFDA}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.06640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>25</v>
       </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{E4003426-26D4-49FB-9D73-933A112A6EE2}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added ElementPage. Test Case,WebTable Testing Add Edit Delete,Added new Utilitiy suitlistiner for safer execution of each row of data.
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joyia\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C646B8E9-7DC9-4D50-9C9D-55AB431CA0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC318221-F69B-4C92-8DEC-6738D00F8794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{1ED0BB6F-46F8-4F2E-967F-0A43B142E062}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="51">
   <si>
     <t>UserName</t>
   </si>
@@ -138,6 +138,60 @@
   </si>
   <si>
     <t>Lorem Ipsum is simply dummy text of the printing and typesetting industry. Lorem Ipsum has been the industry's standard dummy text ever since the 1500s, when an unknown printer took a galley of type and scrambled it to make a type specimen book. It has survived not only five centuries, but also the leap into electronic typesetting, remaining essentially unchanged. It was popularised in the 1960s with the release of Letraset sheets containing Lorem Ipsum passages, and more recently with desktop publishing software like Aldus PageMaker including versions of Lorem Ipsum.</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>69</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>1500000</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>EditFirstName</t>
+  </si>
+  <si>
+    <t>EditLastName</t>
+  </si>
+  <si>
+    <t>EditEmail</t>
+  </si>
+  <si>
+    <t>EditAge</t>
+  </si>
+  <si>
+    <t>EditSalary</t>
+  </si>
+  <si>
+    <t>EditDepartment</t>
+  </si>
+  <si>
+    <t>LUFFY</t>
+  </si>
+  <si>
+    <t>MONKEY</t>
+  </si>
+  <si>
+    <t>test13232@mailinator.com</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>243242</t>
+  </si>
+  <si>
+    <t>IT</t>
   </si>
 </sst>
 </file>
@@ -585,7 +639,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E8F5D29-B261-4791-A884-F5DFAD0642EF}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="9.06640625" style="1"/>
@@ -594,10 +648,16 @@
     <col min="5" max="5" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.9296875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.06640625" style="1"/>
+    <col min="8" max="9" width="9.06640625" style="1"/>
+    <col min="10" max="10" width="10.9296875" style="1" customWidth="1"/>
+    <col min="11" max="12" width="9.06640625" style="1"/>
+    <col min="13" max="13" width="10.06640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="9.06640625" style="1"/>
+    <col min="16" max="16" width="17.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -628,8 +688,35 @@
       <c r="J1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -659,11 +746,39 @@
       </c>
       <c r="J2" s="1" t="s">
         <v>23</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{6570131B-F6A1-4AD3-82A7-02314EC3CC99}"/>
+    <hyperlink ref="P2" r:id="rId2" xr:uid="{A5BEF54C-A35E-40D3-82D6-2B1A6AAB12E4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>